<commit_message>
Add Cypress test for index page validation
</commit_message>
<xml_diff>
--- a/test-cases/bridges-test-cases.xlsx
+++ b/test-cases/bridges-test-cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\Bridges\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6472D18-7C93-44B1-8AF5-AF06C870235E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09AAB48-744D-4046-97C5-165D75252BEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1128" yWindow="1068" windowWidth="10092" windowHeight="8964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -405,9 +405,6 @@
     <t>Verify Cart navigation works</t>
   </si>
   <si>
-    <t>Verify hero section content displayed</t>
-  </si>
-  <si>
     <t>Home page remains displayed</t>
   </si>
   <si>
@@ -420,9 +417,6 @@
     <t>Cart page displayed</t>
   </si>
   <si>
-    <t>Heading, description and images displayed</t>
-  </si>
-  <si>
     <t>Hero verified</t>
   </si>
   <si>
@@ -471,9 +465,6 @@
     <t>Search existing menu item</t>
   </si>
   <si>
-    <t>Pasta displayed in results</t>
-  </si>
-  <si>
     <t>Search completed</t>
   </si>
   <si>
@@ -495,9 +486,6 @@
     <t>Pasta</t>
   </si>
   <si>
-    <t>@#$%</t>
-  </si>
-  <si>
     <t>Search with special characters</t>
   </si>
   <si>
@@ -510,9 +498,6 @@
     <t>Verify product card information</t>
   </si>
   <si>
-    <t>Image, flag, name, price, description, rating displayed</t>
-  </si>
-  <si>
     <t>Card verified</t>
   </si>
   <si>
@@ -550,12 +535,6 @@
   </si>
   <si>
     <t>Verify multiple products added</t>
-  </si>
-  <si>
-    <t>All items added</t>
-  </si>
-  <si>
-    <t>Three items added</t>
   </si>
   <si>
     <t>Item added to cart</t>
@@ -983,6 +962,27 @@
   </si>
   <si>
     <t>Verify order page loads successfully</t>
+  </si>
+  <si>
+    <t>Verify hero section content displayed correctly</t>
+  </si>
+  <si>
+    <t>Heading, description and images displayed correctly</t>
+  </si>
+  <si>
+    <t>Only menu items matching the search keyword are displayed in the results</t>
+  </si>
+  <si>
+    <t>@pasta</t>
+  </si>
+  <si>
+    <t>Image, flag, name, price, description, rating displayed correctly</t>
+  </si>
+  <si>
+    <t>multiple products added</t>
+  </si>
+  <si>
+    <t>multiple quantities added</t>
   </si>
 </sst>
 </file>
@@ -1720,6 +1720,39 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="42" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="42" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="15" fontId="21" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="33" borderId="15" xfId="42" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1746,39 +1779,6 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="42" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="15" fontId="21" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="42" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -2187,102 +2187,102 @@
   <sheetData>
     <row r="1" spans="2:11" ht="5.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="28" t="s">
+      <c r="C2" s="22"/>
+      <c r="D2" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="35" t="s">
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="28" t="s">
+      <c r="C3" s="22"/>
+      <c r="D3" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="27"/>
-      <c r="D4" s="31" t="s">
+      <c r="C4" s="22"/>
+      <c r="D4" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="32" t="s">
+      <c r="C5" s="22"/>
+      <c r="D5" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="27"/>
-      <c r="D6" s="33">
+      <c r="C6" s="22"/>
+      <c r="D6" s="28">
         <v>46192</v>
       </c>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="36"/>
-      <c r="I6" s="36"/>
-      <c r="J6" s="36"/>
-      <c r="K6" s="36"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="27"/>
-      <c r="D7" s="32" t="s">
+      <c r="C7" s="22"/>
+      <c r="D7" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="36"/>
-      <c r="K7" s="36"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="21"/>
     </row>
     <row r="9" spans="2:11" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
@@ -2333,7 +2333,7 @@
       <c r="F10" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="G10" s="34" t="s">
+      <c r="G10" s="18" t="s">
         <v>22</v>
       </c>
       <c r="H10" s="11" t="s">
@@ -2357,12 +2357,12 @@
         <v>111</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>192</v>
-      </c>
-      <c r="G11" s="34" t="s">
+        <v>185</v>
+      </c>
+      <c r="G11" s="18" t="s">
         <v>18</v>
       </c>
       <c r="H11" s="11" t="s">
@@ -2386,16 +2386,16 @@
         <v>114</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>193</v>
-      </c>
-      <c r="G12" s="34" t="s">
+        <v>186</v>
+      </c>
+      <c r="G12" s="18" t="s">
         <v>18</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I12" s="11" t="s">
         <v>106</v>
@@ -2415,16 +2415,16 @@
         <v>115</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>194</v>
-      </c>
-      <c r="G13" s="34" t="s">
+        <v>187</v>
+      </c>
+      <c r="G13" s="18" t="s">
         <v>18</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I13" s="11" t="s">
         <v>35</v>
@@ -2444,16 +2444,16 @@
         <v>116</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>195</v>
-      </c>
-      <c r="G14" s="34" t="s">
+        <v>188</v>
+      </c>
+      <c r="G14" s="18" t="s">
         <v>18</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I14" s="11" t="s">
         <v>34</v>
@@ -2473,16 +2473,16 @@
         <v>117</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="G15" s="34" t="s">
+        <v>189</v>
+      </c>
+      <c r="G15" s="18" t="s">
         <v>18</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I15" s="11" t="s">
         <v>33</v>
@@ -2499,27 +2499,27 @@
         <v>24</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>118</v>
+        <v>270</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="G16" s="34" t="s">
+        <v>190</v>
+      </c>
+      <c r="G16" s="18" t="s">
         <v>18</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>123</v>
+        <v>271</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="J16" s="8"/>
       <c r="K16" s="9"/>
     </row>
-    <row r="17" spans="2:12" ht="45.6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" ht="34.200000000000003" x14ac:dyDescent="0.25">
       <c r="B17" s="7" t="str">
         <f>IF(D17&lt;&gt;"","TC_IDX_"&amp;TEXT(COUNTIF($D$10:D17,"&lt;&gt;"),"000"),"")</f>
         <v>TC_IDX_008</v>
@@ -2528,27 +2528,27 @@
         <v>25</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J17" s="2"/>
       <c r="K17" s="9"/>
     </row>
-    <row r="18" spans="2:12" ht="45.6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" ht="34.200000000000003" x14ac:dyDescent="0.25">
       <c r="B18" s="7" t="str">
         <f>IF(D18&lt;&gt;"","TC_IDX_"&amp;TEXT(COUNTIF($D$10:D18,"&lt;&gt;"),"000"),"")</f>
         <v>TC_IDX_009</v>
@@ -2557,22 +2557,22 @@
         <v>25</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="J18" s="8"/>
       <c r="K18" s="9"/>
@@ -2586,22 +2586,22 @@
         <v>25</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="J19" s="8"/>
       <c r="K19" s="9"/>
@@ -2615,22 +2615,22 @@
         <v>25</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H20" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="I20" s="11" t="s">
         <v>136</v>
-      </c>
-      <c r="I20" s="11" t="s">
-        <v>138</v>
       </c>
       <c r="J20" s="8"/>
       <c r="K20" s="9"/>
@@ -2647,22 +2647,22 @@
         <v>39</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>140</v>
+        <v>272</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="J21" s="8"/>
       <c r="K21" s="9"/>
@@ -2676,22 +2676,22 @@
         <v>39</v>
       </c>
       <c r="D22" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="G22" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="H22" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="E22" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>203</v>
-      </c>
-      <c r="G22" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="H22" s="11" t="s">
-        <v>145</v>
-      </c>
       <c r="I22" s="11" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="J22" s="8"/>
       <c r="K22" s="9"/>
@@ -2705,22 +2705,22 @@
         <v>39</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="G23" s="10" t="s">
         <v>31</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="J23" s="8"/>
       <c r="K23" s="9"/>
@@ -2734,22 +2734,22 @@
         <v>39</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E24" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="G24" s="19" t="s">
+        <v>273</v>
+      </c>
+      <c r="H24" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="F24" s="11" t="s">
-        <v>205</v>
-      </c>
-      <c r="G24" s="37" t="s">
-        <v>148</v>
-      </c>
-      <c r="H24" s="11" t="s">
-        <v>146</v>
-      </c>
       <c r="I24" s="11" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="J24" s="8"/>
       <c r="K24" s="9"/>
@@ -2760,25 +2760,25 @@
         <v>TC_IDX_016</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="G25" s="34" t="s">
+        <v>199</v>
+      </c>
+      <c r="G25" s="18" t="s">
         <v>18</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>153</v>
+        <v>274</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="J25" s="8"/>
       <c r="K25" s="9"/>
@@ -2795,13 +2795,13 @@
         <v>26</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="H26" s="11" t="s">
         <v>32</v>
@@ -2824,16 +2824,16 @@
         <v>28</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="I27" s="11" t="s">
         <v>52</v>
@@ -2850,22 +2850,22 @@
         <v>27</v>
       </c>
       <c r="D28" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="E28" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="G28" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="H28" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="I28" s="11" t="s">
         <v>155</v>
-      </c>
-      <c r="E28" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="F28" s="11" t="s">
-        <v>209</v>
-      </c>
-      <c r="G28" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="H28" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="I28" s="11" t="s">
-        <v>160</v>
       </c>
       <c r="J28" s="8"/>
       <c r="K28" s="9"/>
@@ -2882,16 +2882,16 @@
         <v>29</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="I29" s="11" t="s">
         <v>56</v>
@@ -2908,19 +2908,19 @@
         <v>30</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>168</v>
+        <v>276</v>
       </c>
       <c r="I30" s="11" t="s">
         <v>56</v>
@@ -2937,19 +2937,19 @@
         <v>30</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>167</v>
+        <v>275</v>
       </c>
       <c r="I31" s="11" t="s">
         <v>56</v>
@@ -2963,25 +2963,25 @@
         <v>TC_IDX_023</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="J32" s="2"/>
       <c r="K32" s="9"/>
@@ -2992,25 +2992,25 @@
         <v>TC_IDX_024</v>
       </c>
       <c r="C33" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="I33" s="11" t="s">
         <v>170</v>
-      </c>
-      <c r="D33" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="E33" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="F33" s="11" t="s">
-        <v>214</v>
-      </c>
-      <c r="G33" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="H33" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="I33" s="11" t="s">
-        <v>177</v>
       </c>
       <c r="J33" s="2"/>
       <c r="K33" s="9"/>
@@ -3089,102 +3089,102 @@
   <sheetData>
     <row r="1" spans="2:11" ht="5.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="28" t="s">
+      <c r="C2" s="22"/>
+      <c r="D2" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="18" t="s">
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="31"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="28" t="s">
+      <c r="C3" s="22"/>
+      <c r="D3" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="23"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="34"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="27"/>
-      <c r="D4" s="31" t="s">
+      <c r="C4" s="22"/>
+      <c r="D4" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="23"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="33"/>
+      <c r="K4" s="34"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="32" t="s">
+      <c r="C5" s="22"/>
+      <c r="D5" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="21"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="23"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="33"/>
+      <c r="K5" s="34"/>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="27"/>
-      <c r="D6" s="33">
+      <c r="C6" s="22"/>
+      <c r="D6" s="28">
         <v>46192</v>
       </c>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="23"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="34"/>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="27"/>
-      <c r="D7" s="32" t="s">
+      <c r="C7" s="22"/>
+      <c r="D7" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="26"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="36"/>
+      <c r="K7" s="37"/>
     </row>
     <row r="9" spans="2:11" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
@@ -3227,22 +3227,22 @@
         <v>21</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>18</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="J10" s="8"/>
       <c r="K10" s="9"/>
@@ -3256,19 +3256,19 @@
         <v>110</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="E11" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="F11" s="14" t="s">
         <v>184</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>191</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>18</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="I11" s="14" t="s">
         <v>113</v>
@@ -3285,22 +3285,22 @@
         <v>110</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="J12" s="8"/>
       <c r="K12" s="9"/>
@@ -3311,25 +3311,25 @@
         <v>TC_CHK_004</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>18</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="J13" s="8"/>
       <c r="K13" s="9"/>
@@ -3343,7 +3343,7 @@
         <v>63</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="E14" s="14" t="s">
         <v>41</v>
@@ -3372,7 +3372,7 @@
         <v>63</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="E15" s="14" t="s">
         <v>42</v>
@@ -3401,7 +3401,7 @@
         <v>63</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E16" s="14" t="s">
         <v>49</v>
@@ -3413,10 +3413,10 @@
         <v>45</v>
       </c>
       <c r="H16" s="16" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="J16" s="8"/>
       <c r="K16" s="9"/>
@@ -3430,19 +3430,19 @@
         <v>63</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>41</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="G17" s="14" t="s">
         <v>51</v>
       </c>
       <c r="H17" s="16" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="I17" s="14" t="s">
         <v>52</v>
@@ -3485,7 +3485,7 @@
         <v>TC_CHK_010</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>57</v>
@@ -3514,25 +3514,25 @@
         <v>TC_CHK_011</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>58</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="H20" s="14" t="s">
         <v>62</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J20" s="8"/>
       <c r="K20" s="9"/>
@@ -3543,25 +3543,25 @@
         <v>TC_CHK_012</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="E21" s="14" t="s">
         <v>58</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="H21" s="14" t="s">
         <v>62</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J21" s="8"/>
       <c r="K21" s="9"/>
@@ -3572,25 +3572,25 @@
         <v>TC_CHK_013</v>
       </c>
       <c r="C22" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="D22" s="14" t="s">
         <v>229</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>236</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>58</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="H22" s="14" t="s">
         <v>62</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J22" s="8"/>
       <c r="K22" s="9"/>
@@ -3601,25 +3601,25 @@
         <v>TC_CHK_014</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>58</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="H23" s="14" t="s">
         <v>62</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J23" s="8"/>
       <c r="K23" s="9"/>
@@ -3630,7 +3630,7 @@
         <v>TC_CHK_015</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D24" s="14" t="s">
         <v>77</v>
@@ -3659,7 +3659,7 @@
         <v>TC_CHK_016</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D25" s="14" t="s">
         <v>65</v>
@@ -3677,7 +3677,7 @@
         <v>67</v>
       </c>
       <c r="I25" s="14" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="J25" s="2"/>
       <c r="K25" s="9"/>
@@ -3688,7 +3688,7 @@
         <v>TC_CHK_017</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>68</v>
@@ -3700,10 +3700,10 @@
         <v>69</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="I26" s="14" t="s">
         <v>71</v>
@@ -3717,7 +3717,7 @@
         <v>TC_CHK_018</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>72</v>
@@ -3749,7 +3749,7 @@
         <v>82</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="E28" s="14" t="s">
         <v>40</v>
@@ -3761,10 +3761,10 @@
         <v>84</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="J28" s="8"/>
       <c r="K28" s="9"/>
@@ -3790,10 +3790,10 @@
         <v>88</v>
       </c>
       <c r="H29" s="14" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="J29" s="8"/>
       <c r="K29" s="9"/>
@@ -3869,102 +3869,102 @@
   <sheetData>
     <row r="1" spans="2:11" ht="5.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="28" t="s">
+      <c r="C2" s="22"/>
+      <c r="D2" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="18" t="s">
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="29" t="s">
         <v>105</v>
       </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="31"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="28" t="s">
+      <c r="C3" s="22"/>
+      <c r="D3" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="23"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="34"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="27"/>
-      <c r="D4" s="31" t="s">
+      <c r="C4" s="22"/>
+      <c r="D4" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="23"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="33"/>
+      <c r="K4" s="34"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="32" t="s">
+      <c r="C5" s="22"/>
+      <c r="D5" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="21"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="23"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="33"/>
+      <c r="K5" s="34"/>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="27"/>
-      <c r="D6" s="33">
+      <c r="C6" s="22"/>
+      <c r="D6" s="28">
         <v>46192</v>
       </c>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="23"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="34"/>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="27"/>
-      <c r="D7" s="32" t="s">
+      <c r="C7" s="22"/>
+      <c r="D7" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="26"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="36"/>
+      <c r="K7" s="37"/>
     </row>
     <row r="9" spans="2:11" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
@@ -4007,22 +4007,22 @@
         <v>21</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>18</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J10" s="8"/>
       <c r="K10" s="9"/>
@@ -4042,7 +4042,7 @@
         <v>90</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>18</v>
@@ -4062,25 +4062,25 @@
         <v>TC_ORD_003</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>98</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="J12" s="8"/>
       <c r="K12" s="9"/>
@@ -4091,13 +4091,13 @@
         <v>TC_ORD_004</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="F13" s="11" t="s">
         <v>92</v>
@@ -4106,10 +4106,10 @@
         <v>98</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="J13" s="8"/>
       <c r="K13" s="9"/>
@@ -4120,13 +4120,13 @@
         <v>TC_ORD_005</v>
       </c>
       <c r="C14" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="D14" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="D14" s="11" t="s">
-        <v>260</v>
-      </c>
       <c r="E14" s="11" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="F14" s="11" t="s">
         <v>93</v>
@@ -4138,7 +4138,7 @@
         <v>94</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="J14" s="8"/>
       <c r="K14" s="9"/>
@@ -4149,16 +4149,16 @@
         <v>TC_ORD_006</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>95</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>98</v>
@@ -4167,7 +4167,7 @@
         <v>96</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="J15" s="8"/>
       <c r="K15" s="9"/>
@@ -4178,13 +4178,13 @@
         <v>TC_ORD_007</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="F16" s="11" t="s">
         <v>97</v>
@@ -4193,10 +4193,10 @@
         <v>98</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="J16" s="8"/>
       <c r="K16" s="9"/>
@@ -4207,16 +4207,16 @@
         <v>TC_ORD_008</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>99</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="G17" s="10" t="s">
         <v>98</v>
@@ -4225,7 +4225,7 @@
         <v>100</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="J17" s="8"/>
       <c r="K17" s="9"/>
@@ -4236,13 +4236,13 @@
         <v>TC_ORD_009</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="F18" s="11" t="s">
         <v>101</v>
@@ -4265,13 +4265,13 @@
         <v>TC_ORD_010</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>101</v>
@@ -4280,10 +4280,10 @@
         <v>102</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="J19" s="8"/>
       <c r="K19" s="9"/>

</xml_diff>